<commit_message>
Update README clone URL and run command
Replace the placeholder clone URL with the actual repository URL (https://github.com/kasun28/Playwright-project) and simplify the example python command by removing extra flags. Also update the 'Assignment 1 - Test cases.xlsx' file (binary contents changed). These edits clarify how to clone the repo and run the automation with the minimal example command.
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -458,7 +458,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -577,7 +577,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>ඔයාගෙ අම්මගෙන් අනුමැතිය ගත්තද?</t>
+          <t>ඔයාගෙ අම්මගෙන් අනුමතිය ගත්තද?</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">

</xml_diff>